<commit_message>
update: Update rules for identify day, year and month
</commit_message>
<xml_diff>
--- a/detectors/qty/dataset/dataset.xlsx
+++ b/detectors/qty/dataset/dataset.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\codes\nl2sql\detectors\qty\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B6327D-9768-4F46-9201-75CE205C3704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84180A63-B4E9-438D-92B5-6D868F9EC02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="353">
   <si>
     <t>id</t>
   </si>
@@ -544,304 +545,541 @@
     <t>2025-04-01 ; 2025-04-30</t>
   </si>
   <si>
+    <t>3 akun</t>
+  </si>
+  <si>
+    <t>30 hari</t>
+  </si>
+  <si>
+    <t>5.000.000</t>
+  </si>
+  <si>
+    <t>7 transaksi;2025</t>
+  </si>
+  <si>
+    <t>10 transaksi</t>
+  </si>
+  <si>
+    <t>90 hari</t>
+  </si>
+  <si>
+    <t>1.000.000; 10.000.000 rupiah</t>
+  </si>
+  <si>
+    <t>1.000.000</t>
+  </si>
+  <si>
+    <t>50.000.000</t>
+  </si>
+  <si>
+    <t>10.000</t>
+  </si>
+  <si>
+    <t>7 laporan</t>
+  </si>
+  <si>
+    <t>bulan</t>
+  </si>
+  <si>
+    <t>60 hari</t>
+  </si>
+  <si>
+    <t>20.000.000; 100.000.000</t>
+  </si>
+  <si>
+    <t>5 pengiriman;10 Mei 2025</t>
+  </si>
+  <si>
+    <t>10 unit</t>
+  </si>
+  <si>
+    <t>7 pengiriman;2025</t>
+  </si>
+  <si>
+    <t>3 rute</t>
+  </si>
+  <si>
+    <t>100 unit</t>
+  </si>
+  <si>
+    <t>10 detail</t>
+  </si>
+  <si>
+    <t>5 supir</t>
+  </si>
+  <si>
+    <t>100 km</t>
+  </si>
+  <si>
+    <t>14 hari</t>
+  </si>
+  <si>
+    <t>2000 kg</t>
+  </si>
+  <si>
+    <t>10 pengiriman</t>
+  </si>
+  <si>
+    <t>7 kendaraan</t>
+  </si>
+  <si>
+    <t>April 2025</t>
+  </si>
+  <si>
+    <t>5000 km</t>
+  </si>
+  <si>
+    <t>10 supir</t>
+  </si>
+  <si>
+    <t>1  Mei 2025</t>
+  </si>
+  <si>
+    <t>5 pemasok</t>
+  </si>
+  <si>
+    <t>2025-04-01 ; 2025-04-15</t>
+  </si>
+  <si>
+    <t>3 pembelian</t>
+  </si>
+  <si>
+    <t>Selasa</t>
+  </si>
+  <si>
+    <t>7 barang</t>
+  </si>
+  <si>
+    <t>50 unit</t>
+  </si>
+  <si>
+    <t>1 Mei 2025</t>
+  </si>
+  <si>
+    <t>5 vendor</t>
+  </si>
+  <si>
+    <t>2025-04-01; 2025-04-30</t>
+  </si>
+  <si>
+    <t>3 barang</t>
+  </si>
+  <si>
+    <t>100.000.000</t>
+  </si>
+  <si>
+    <t>200 unit</t>
+  </si>
+  <si>
+    <t>7 pengadaan;2025</t>
+  </si>
+  <si>
+    <t>1 Januari 2025</t>
+  </si>
+  <si>
+    <t>5 penilaian</t>
+  </si>
+  <si>
+    <t>2025-04-01</t>
+  </si>
+  <si>
+    <t>5 Mei 2025</t>
+  </si>
+  <si>
+    <t>3 vendor</t>
+  </si>
+  <si>
+    <t>100 karakter</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 penilaian;2025 </t>
+  </si>
+  <si>
+    <t>10 per transaksi</t>
+  </si>
+  <si>
+    <t>2025-04-15;2025-04-30;100unit</t>
+  </si>
+  <si>
+    <t>10 transaksi;10 Mei 2025</t>
+  </si>
+  <si>
+    <t>20;50 unit</t>
+  </si>
+  <si>
+    <t>7 transaksi</t>
+  </si>
+  <si>
+    <t>5 feedback</t>
+  </si>
+  <si>
+    <t>10 komentar</t>
+  </si>
+  <si>
+    <t>Januari 2025</t>
+  </si>
+  <si>
+    <t>3 pelanggan</t>
+  </si>
+  <si>
+    <t>2 kali</t>
+  </si>
+  <si>
+    <t>minggu</t>
+  </si>
+  <si>
+    <t>7 feedback</t>
+  </si>
+  <si>
+    <t>5 produksi;9 Mei 2025</t>
+  </si>
+  <si>
+    <t>10 kali;minggu</t>
+  </si>
+  <si>
+    <t>3 produk</t>
+  </si>
+  <si>
+    <t>5000 unit</t>
+  </si>
+  <si>
+    <t>7 detail</t>
+  </si>
+  <si>
+    <t>1000 unit</t>
+  </si>
+  <si>
+    <t>5 detail;100 unit</t>
+  </si>
+  <si>
+    <t>200 kali</t>
+  </si>
+  <si>
+    <t>3 perencanaan</t>
+  </si>
+  <si>
+    <t>7 bahan baku</t>
+  </si>
+  <si>
+    <t>keuangan.json</t>
+  </si>
+  <si>
+    <t>logistik.json</t>
+  </si>
+  <si>
+    <t>pembelian.json</t>
+  </si>
+  <si>
+    <t>pengadaan.json</t>
+  </si>
+  <si>
+    <t>penjualan.json</t>
+  </si>
+  <si>
+    <t>produksi.json</t>
+  </si>
+  <si>
+    <t>Berapa total unit yang diproduksi oleh mesin tipe A pada tanggal 5 Januari 2024 dalam satu hari?</t>
+  </si>
+  <si>
+    <t>Selama bulan Maret 2025, berapa kali mesin tipe B memproduksi lebih dari 1000 unit per hari?</t>
+  </si>
+  <si>
+    <t>Berapa jumlah produksi harian untuk produk "Sabun Cair" selama 7 hari pertama bulan April 2023?</t>
+  </si>
+  <si>
+    <t>Pada minggu ketiga bulan Juni 2024, mesin dengan kapasitas di atas 500 unit memproduksi berapa total unit per hari?</t>
+  </si>
+  <si>
+    <t>Berapa kali mesin tipe C memproduksi produk "Pasta Gigi" dalam seminggu penuh di bulan Februari 2023?</t>
+  </si>
+  <si>
+    <t>Total produksi produk "Minyak Goreng" dari tanggal 1 sampai 10 Desember 2024 oleh mesin tipe D per hari berapa?</t>
+  </si>
+  <si>
+    <t>Selama tiga bulan pertama tahun 2025, berapa banyak mesin yang menghasilkan lebih dari 500 unit dalam satu hari?</t>
+  </si>
+  <si>
+    <t>Berapa rata-rata jumlah produksi per hari untuk produk "Sampo" selama bulan Juli dan Agustus 2023?</t>
+  </si>
+  <si>
+    <t>Dalam 30 hari terakhir dari tahun 2024, mesin tipe B memproduksi berapa total unit dan berapa kali?</t>
+  </si>
+  <si>
+    <t>Berapa jumlah total produksi mingguan untuk produk "Pasta Gigi" selama tahun 2023 oleh mesin berkapasitas di atas 1000 unit?</t>
+  </si>
+  <si>
+    <t>5 Januari 2024; satu hari</t>
+  </si>
+  <si>
+    <t>seminggu penuh; Februari 2023</t>
+  </si>
+  <si>
+    <t>1;10 Desember 2024; produksi total; per hari</t>
+  </si>
+  <si>
+    <t>1.000.000 rupiah</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Kalimat</t>
+  </si>
+  <si>
+    <t>Frasa Kuantitas</t>
+  </si>
+  <si>
+    <t>per hari</t>
+  </si>
+  <si>
+    <t>akhir pekan</t>
+  </si>
+  <si>
+    <t>gudang.json</t>
+  </si>
+  <si>
+    <t>Berapa jumlah barang yang masuk pada tanggal 5 Mei 2024?</t>
+  </si>
+  <si>
+    <t>Tampilkan transaksi keluar pada bulan Januari 2023.</t>
+  </si>
+  <si>
+    <t>Barang apa saja yang keluar pada tanggal 1 Maret 2025?</t>
+  </si>
+  <si>
+    <t>Ada berapa transaksi yang terjadi pada hari Senin, 10 Juni 2024?</t>
+  </si>
+  <si>
+    <t>Total barang yang masuk selama tahun 2022 berapa?</t>
+  </si>
+  <si>
+    <t>Siapa saja pelanggan yang bertransaksi pada tanggal 12 Desember 2023?</t>
+  </si>
+  <si>
+    <t>Apa produk yang paling banyak dibeli pada bulan Februari 2025?</t>
+  </si>
+  <si>
+    <t>Berapa total harga transaksi pada tanggal 14 Februari 2024?</t>
+  </si>
+  <si>
+    <t>Tampilkan semua transaksi yang terjadi pada tahun 2023.</t>
+  </si>
+  <si>
+    <t>Transaksi masuk apa saja yang terjadi pada hari Kamis, 7 Maret 2024?</t>
+  </si>
+  <si>
+    <t>Barang apa yang memiliki stok lebih dari 100 unit?</t>
+  </si>
+  <si>
+    <t>Tampilkan produk dengan harga di atas 50000.</t>
+  </si>
+  <si>
+    <t>Ada berapa produk dengan jumlah diskon lebih dari 10%?</t>
+  </si>
+  <si>
+    <t>Gudang mana yang menyimpan lebih dari 200 item?</t>
+  </si>
+  <si>
+    <t>Tampilkan barang yang pernah keluar sebanyak 50 unit atau lebih.</t>
+  </si>
+  <si>
+    <t>Ada berapa barang dengan satuan "kg" dan stok di bawah 20?</t>
+  </si>
+  <si>
+    <t>Produk dengan harga antara 10000 dan 30000 apa saja?</t>
+  </si>
+  <si>
+    <t>Tampilkan total jumlah barang yang keluar dari gudang utama.</t>
+  </si>
+  <si>
+    <t>Ada berapa kategori barang dengan lebih dari 5 jenis barang?</t>
+  </si>
+  <si>
+    <t>Produk apa yang memiliki total jumlah pembelian lebih dari 300?</t>
+  </si>
+  <si>
+    <t>Berapa banyak transaksi yang terjadi setiap hari Jumat?</t>
+  </si>
+  <si>
+    <t>Tampilkan barang yang paling sering masuk setiap hari Senin.</t>
+  </si>
+  <si>
+    <t>Hari apa yang paling banyak terjadi transaksi keluar?</t>
+  </si>
+  <si>
+    <t>Berapa jumlah rata-rata barang masuk per hari?</t>
+  </si>
+  <si>
+    <t>Barang apa yang paling sering keluar dalam seminggu terakhir?</t>
+  </si>
+  <si>
+    <t>Tampilkan semua transaksi yang terjadi pada akhir pekan.</t>
+  </si>
+  <si>
+    <t>Berapa kali pelanggan dengan nama Budi melakukan transaksi dalam seminggu?</t>
+  </si>
+  <si>
+    <t>Tampilkan tanggal-tanggal di mana terjadi lebih dari 3 transaksi.</t>
+  </si>
+  <si>
+    <t>Produk apa yang paling banyak dibeli dalam satu minggu terakhir?</t>
+  </si>
+  <si>
+    <t>Kapan terakhir kali terjadi transaksi masuk?</t>
+  </si>
+  <si>
+    <t>5 Mei 2024</t>
+  </si>
+  <si>
+    <t>1 Maret 2025</t>
+  </si>
+  <si>
+    <t>Senin, 10 Juni 2024</t>
+  </si>
+  <si>
+    <t>12 Desember 2023</t>
+  </si>
+  <si>
+    <t>14 Februari 2024</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>10%</t>
+  </si>
+  <si>
+    <t>200 item</t>
+  </si>
+  <si>
+    <t>20 kg</t>
+  </si>
+  <si>
+    <t>10000;30000</t>
+  </si>
+  <si>
+    <t>5 jenis</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>satu minggu terakhir</t>
+  </si>
+  <si>
+    <t>3 transaksi</t>
+  </si>
+  <si>
+    <t>seminggu</t>
+  </si>
+  <si>
+    <t>seminggu terakhir</t>
+  </si>
+  <si>
+    <t>bulanJanuari 2023</t>
+  </si>
+  <si>
     <t>April</t>
   </si>
   <si>
-    <t>3 akun</t>
+    <t>Mei 2025</t>
+  </si>
+  <si>
+    <t>Januari;Maret 2025</t>
+  </si>
+  <si>
+    <t>Maret 2025</t>
+  </si>
+  <si>
+    <t>5 kali; April 2025</t>
+  </si>
+  <si>
+    <t>5 produk;April 2025</t>
+  </si>
+  <si>
+    <t>3 pelanggan;April</t>
+  </si>
+  <si>
+    <t>10%;Mei 2025</t>
+  </si>
+  <si>
+    <t>Maret 2025; 1000 unit</t>
+  </si>
+  <si>
+    <t>minggu ketiga; Juni 2024; 500 unit</t>
+  </si>
+  <si>
+    <t>Juli; Agustus 2023</t>
+  </si>
+  <si>
+    <t>Februari 2025</t>
   </si>
   <si>
     <t>Senin;minggu</t>
   </si>
   <si>
-    <t>30 hari</t>
-  </si>
-  <si>
-    <t>5.000.000</t>
-  </si>
-  <si>
-    <t>7 transaksi;2025</t>
-  </si>
-  <si>
-    <t>10 transaksi</t>
-  </si>
-  <si>
-    <t>90 hari</t>
-  </si>
-  <si>
-    <t>1.000.000; 10.000.000 rupiah</t>
-  </si>
-  <si>
-    <t>Mei 2025</t>
-  </si>
-  <si>
-    <t>Januari;Maret 2025</t>
-  </si>
-  <si>
-    <t>1.000.000</t>
-  </si>
-  <si>
-    <t>50.000.000</t>
-  </si>
-  <si>
-    <t>10.000</t>
-  </si>
-  <si>
-    <t>7 laporan</t>
-  </si>
-  <si>
-    <t>bulan</t>
-  </si>
-  <si>
-    <t>60 hari</t>
-  </si>
-  <si>
-    <t>20.000.000; 100.000.000</t>
-  </si>
-  <si>
-    <t>5 pengiriman;10 Mei 2025</t>
-  </si>
-  <si>
     <t>3 pengiriman;Senin</t>
   </si>
   <si>
-    <t>10 unit</t>
-  </si>
-  <si>
-    <t>7 pengiriman;2025</t>
+    <t>Rabu;minggu</t>
+  </si>
+  <si>
+    <t>Rabu</t>
+  </si>
+  <si>
+    <t>3 kali;sabtu</t>
+  </si>
+  <si>
+    <t>Senin;Rabu</t>
+  </si>
+  <si>
+    <t>7 pertama; April 2023</t>
+  </si>
+  <si>
+    <t>Kamis, 7 Maret 2024</t>
+  </si>
+  <si>
+    <t>Jumat</t>
+  </si>
+  <si>
+    <t>Senin</t>
+  </si>
+  <si>
+    <t>2024</t>
   </si>
   <si>
     <t>50 kali;2024</t>
   </si>
   <si>
-    <t>3 rute</t>
-  </si>
-  <si>
-    <t>Rabu;minggu</t>
-  </si>
-  <si>
-    <t>100 unit</t>
-  </si>
-  <si>
-    <t>1 Januai 2025</t>
-  </si>
-  <si>
-    <t>10 detail</t>
-  </si>
-  <si>
-    <t>5 supir</t>
-  </si>
-  <si>
-    <t>tahun 2024</t>
-  </si>
-  <si>
-    <t>100 km</t>
-  </si>
-  <si>
-    <t>14 hari</t>
-  </si>
-  <si>
-    <t>2000 kg</t>
-  </si>
-  <si>
-    <t>10 pengiriman</t>
-  </si>
-  <si>
-    <t>7 kendaraan</t>
-  </si>
-  <si>
-    <t>April 2025</t>
-  </si>
-  <si>
-    <t>5000 km</t>
-  </si>
-  <si>
-    <t>10 supir</t>
-  </si>
-  <si>
-    <t>1  Mei 2025</t>
-  </si>
-  <si>
-    <t>5 pemasok</t>
-  </si>
-  <si>
-    <t>2025-04-01 ; 2025-04-15</t>
-  </si>
-  <si>
     <t>10 kali; 2024</t>
   </si>
   <si>
-    <t>Maret 2025</t>
-  </si>
-  <si>
-    <t>3 pembelian</t>
-  </si>
-  <si>
-    <t>Selasa</t>
-  </si>
-  <si>
-    <t>7 barang</t>
-  </si>
-  <si>
-    <t>50 unit</t>
-  </si>
-  <si>
-    <t>1 Mei 2025</t>
-  </si>
-  <si>
-    <t>5 vendor</t>
-  </si>
-  <si>
-    <t>2025-04-01; 2025-04-30</t>
-  </si>
-  <si>
-    <t>3 barang</t>
-  </si>
-  <si>
-    <t>100.000.000</t>
-  </si>
-  <si>
-    <t>5 kali; April 2025</t>
-  </si>
-  <si>
-    <t>200 unit</t>
-  </si>
-  <si>
-    <t>7 pengadaan;2025</t>
-  </si>
-  <si>
-    <t>1 Januari 2025</t>
-  </si>
-  <si>
-    <t>5 penilaian</t>
-  </si>
-  <si>
-    <t>2025-04-01</t>
-  </si>
-  <si>
-    <t>5 Mei 2025</t>
-  </si>
-  <si>
-    <t>3 vendor</t>
-  </si>
-  <si>
-    <t>100 karakter</t>
-  </si>
-  <si>
-    <t>3.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 penilaian;2025 </t>
-  </si>
-  <si>
-    <t>Rabu</t>
-  </si>
-  <si>
-    <t>5 produk;April 2025</t>
-  </si>
-  <si>
-    <t>3 kali;sabtu</t>
-  </si>
-  <si>
-    <t>10 per transaksi</t>
-  </si>
-  <si>
-    <t>2025-04-15;2025-04-30;100unit</t>
-  </si>
-  <si>
-    <t>10 transaksi;10 Mei 2025</t>
-  </si>
-  <si>
     <t>500 unit;2024</t>
   </si>
   <si>
-    <t>3 pelanggan;April</t>
-  </si>
-  <si>
-    <t>20;50 unit</t>
-  </si>
-  <si>
-    <t>10%;Mei 2025</t>
-  </si>
-  <si>
-    <t>7 transaksi</t>
-  </si>
-  <si>
-    <t>5 feedback</t>
-  </si>
-  <si>
-    <t>10 komentar</t>
-  </si>
-  <si>
-    <t>Januari 2025</t>
-  </si>
-  <si>
-    <t>Senin;Rabu</t>
-  </si>
-  <si>
-    <t>3 pelanggan</t>
-  </si>
-  <si>
-    <t>2 kali</t>
-  </si>
-  <si>
-    <t>minggu</t>
-  </si>
-  <si>
-    <t>7 feedback</t>
-  </si>
-  <si>
-    <t>5 produksi;9 Mei 2025</t>
-  </si>
-  <si>
-    <t>10 kali;minggu</t>
-  </si>
-  <si>
-    <t>3 produk</t>
-  </si>
-  <si>
-    <t>5000 unit</t>
-  </si>
-  <si>
-    <t>7 detail</t>
-  </si>
-  <si>
-    <t>1000 unit</t>
-  </si>
-  <si>
     <t>10 produksi;2025</t>
   </si>
   <si>
-    <t>5 detail;100 unit</t>
-  </si>
-  <si>
-    <t>200 kali</t>
-  </si>
-  <si>
-    <t>3 perencanaan</t>
-  </si>
-  <si>
-    <t>7 bahan baku</t>
-  </si>
-  <si>
     <t>10 perencanaan;2025</t>
   </si>
   <si>
-    <t>keuangan.json</t>
-  </si>
-  <si>
-    <t>logistik.json</t>
-  </si>
-  <si>
-    <t>pembelian.json</t>
-  </si>
-  <si>
-    <t>pengadaan.json</t>
-  </si>
-  <si>
-    <t>penjualan.json</t>
-  </si>
-  <si>
-    <t>produksi.json</t>
+    <t>tiga pertama; 2025; 500 unit; satu hari</t>
+  </si>
+  <si>
+    <t>30 hari; 2024</t>
+  </si>
+  <si>
+    <t>mingguan; 2023; 1000 unit</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>2023</t>
   </si>
 </sst>
 </file>
@@ -903,12 +1141,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1213,10 +1468,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F206"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="67.7265625" customWidth="1"/>
+    <col min="2" max="2" width="45.453125" style="4" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="36.81640625" customWidth="1"/>
@@ -1227,7 +1482,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1247,25 +1502,25 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>268</v>
-      </c>
-      <c r="E2" s="2">
-        <v>45778</v>
+        <v>247</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E3" t="s">
         <v>171</v>
@@ -1275,11 +1530,11 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E4" t="s">
         <v>172</v>
@@ -1289,11 +1544,11 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E5" t="s">
         <v>173</v>
@@ -1303,176 +1558,176 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E6" t="s">
-        <v>174</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E8" t="s">
-        <v>176</v>
+        <v>332</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="4" t="s">
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>268</v>
-      </c>
-      <c r="E10">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>247</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E11" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="4" t="s">
         <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E15" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E16" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E17" t="s">
-        <v>183</v>
+        <v>321</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E18">
         <v>2024</v>
@@ -1482,72 +1737,72 @@
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="4" t="s">
         <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E20" t="s">
-        <v>184</v>
+        <v>322</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E23" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="4" t="s">
         <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E24">
         <v>2025</v>
@@ -1557,165 +1812,162 @@
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E25" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="4" t="s">
         <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E26" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E27" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="4" t="s">
         <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E28" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>268</v>
-      </c>
-      <c r="E29" t="s">
-        <v>189</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C30" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E30" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C31" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="E31" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>1</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C32" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E32" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C33" t="s">
-        <v>269</v>
-      </c>
-      <c r="E33" s="2">
-        <v>45748</v>
+        <v>248</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>3</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C34" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E34" t="s">
-        <v>193</v>
+        <v>333</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>4</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E35" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>5</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E36" t="s">
         <v>173</v>
@@ -1725,791 +1977,791 @@
       <c r="A37">
         <v>6</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="4" t="s">
         <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>7</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E38" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>8</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="4" t="s">
         <v>43</v>
       </c>
       <c r="C39" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E39" t="s">
-        <v>196</v>
+        <v>343</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>9</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="4" t="s">
         <v>44</v>
       </c>
       <c r="C40" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E40" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>10</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C41" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E41" t="s">
-        <v>198</v>
+        <v>334</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>11</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="4" t="s">
         <v>46</v>
       </c>
       <c r="C42" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E42" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>12</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="4" t="s">
         <v>47</v>
       </c>
       <c r="C43" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E43" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>13</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="4" t="s">
         <v>48</v>
       </c>
       <c r="C44" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E44" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>14</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="4" t="s">
         <v>49</v>
       </c>
       <c r="C45" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E45" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>15</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="4" t="s">
         <v>50</v>
       </c>
       <c r="C46" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E46" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>16</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="4" t="s">
         <v>51</v>
       </c>
       <c r="C47" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E47" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>17</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="4" t="s">
         <v>52</v>
       </c>
       <c r="C48" t="s">
-        <v>269</v>
-      </c>
-      <c r="E48" t="s">
-        <v>203</v>
+        <v>248</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>18</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="4" t="s">
         <v>53</v>
       </c>
       <c r="C49" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E49" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>19</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C50" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E50" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>20</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C51" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E51" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>21</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C52" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>22</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="4" t="s">
         <v>57</v>
       </c>
       <c r="C53" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E53" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>23</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="4" t="s">
         <v>58</v>
       </c>
       <c r="C54" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E54" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>24</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C55" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E55" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>25</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C56" t="s">
-        <v>269</v>
-      </c>
-      <c r="E56" t="s">
-        <v>209</v>
+        <v>248</v>
+      </c>
+      <c r="E56" s="9">
+        <v>45748</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>26</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C57" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E57" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>27</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="4" t="s">
         <v>62</v>
       </c>
       <c r="C58" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E58" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>28</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="4" t="s">
         <v>63</v>
       </c>
       <c r="C59" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E59" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>29</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="4" t="s">
         <v>64</v>
       </c>
       <c r="C60" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>30</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="4" t="s">
         <v>65</v>
       </c>
       <c r="C61" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="E61" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>1</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="4" t="s">
         <v>66</v>
       </c>
       <c r="C62" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E62" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>2</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C63" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E63" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>3</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="4" t="s">
         <v>68</v>
       </c>
       <c r="C64" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E64" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>4</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="4" t="s">
         <v>69</v>
       </c>
       <c r="C65" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>5</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C66" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E66" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>6</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="4" t="s">
         <v>71</v>
       </c>
       <c r="C67" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E67" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>7</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="4" t="s">
         <v>72</v>
       </c>
       <c r="C68" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E68" t="s">
-        <v>215</v>
+        <v>344</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>8</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="4" t="s">
         <v>73</v>
       </c>
       <c r="C69" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E69" t="s">
-        <v>216</v>
+        <v>323</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>9</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C70" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E70" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>10</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C71" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E71" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>11</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="4" t="s">
         <v>76</v>
       </c>
       <c r="C72" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E72" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>12</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="4" t="s">
         <v>77</v>
       </c>
       <c r="C73" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E73" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>13</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C74" t="s">
-        <v>270</v>
-      </c>
-      <c r="E74">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+        <v>249</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>14</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="4" t="s">
         <v>79</v>
       </c>
       <c r="C75" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E75" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>15</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="4" t="s">
         <v>80</v>
       </c>
       <c r="C76" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="E76" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>1</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="4" t="s">
         <v>81</v>
       </c>
       <c r="C77" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E77" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>2</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C78" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E78" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>3</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="4" t="s">
         <v>83</v>
       </c>
       <c r="C79" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E79" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>4</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C80" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E80" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>5</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="4" t="s">
         <v>85</v>
       </c>
       <c r="C81" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>6</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="4" t="s">
         <v>86</v>
       </c>
       <c r="C82" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E82" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>7</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="4" t="s">
         <v>87</v>
       </c>
       <c r="C83" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E83" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>8</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C84" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E84" t="s">
-        <v>226</v>
+        <v>324</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>9</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="4" t="s">
         <v>89</v>
       </c>
       <c r="C85" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E85" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>10</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="4" t="s">
         <v>90</v>
       </c>
       <c r="C86" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E86" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>11</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="4" t="s">
         <v>91</v>
       </c>
       <c r="C87" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E87" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>12</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="4" t="s">
         <v>92</v>
       </c>
       <c r="C88" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E88" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>13</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="4" t="s">
         <v>93</v>
       </c>
       <c r="C89" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>14</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="4" t="s">
         <v>94</v>
       </c>
       <c r="C90" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E90" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>15</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="4" t="s">
         <v>95</v>
       </c>
       <c r="C91" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E91" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>16</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="4" t="s">
         <v>96</v>
       </c>
       <c r="C92" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E92" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>17</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="4" t="s">
         <v>97</v>
       </c>
       <c r="C93" t="s">
-        <v>271</v>
-      </c>
-      <c r="E93" t="s">
-        <v>209</v>
+        <v>250</v>
+      </c>
+      <c r="E93" s="9">
+        <v>45748</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>18</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C94" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E94">
         <v>4</v>
@@ -2519,81 +2771,81 @@
       <c r="A95">
         <v>19</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="4" t="s">
         <v>99</v>
       </c>
       <c r="C95" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E95" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>20</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="4" t="s">
         <v>100</v>
       </c>
       <c r="C96" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E96" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>21</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="4" t="s">
         <v>101</v>
       </c>
       <c r="C97" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E97" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>22</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="4" t="s">
         <v>102</v>
       </c>
       <c r="C98" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E98" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>23</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="4" t="s">
         <v>103</v>
       </c>
       <c r="C99" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E99" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>24</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="4" t="s">
         <v>104</v>
       </c>
       <c r="C100" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E100">
         <v>2024</v>
@@ -2603,11 +2855,11 @@
       <c r="A101">
         <v>25</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="4" t="s">
         <v>105</v>
       </c>
       <c r="C101" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E101">
         <v>2</v>
@@ -2617,64 +2869,64 @@
       <c r="A102">
         <v>26</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="4" t="s">
         <v>106</v>
       </c>
       <c r="C102" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E102" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>27</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="4" t="s">
         <v>107</v>
       </c>
       <c r="C103" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E103" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>28</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="4" t="s">
         <v>108</v>
       </c>
       <c r="C104" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>29</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="4" t="s">
         <v>109</v>
       </c>
       <c r="C105" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E105" t="s">
-        <v>237</v>
+        <v>335</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>30</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="4" t="s">
         <v>110</v>
       </c>
       <c r="C106" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E106">
         <v>5</v>
@@ -2684,484 +2936,484 @@
       <c r="A107">
         <v>1</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="4" t="s">
         <v>111</v>
       </c>
       <c r="C107" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E107" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>2</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="4" t="s">
         <v>112</v>
       </c>
       <c r="C108" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E108" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>3</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="4" t="s">
         <v>113</v>
       </c>
       <c r="C109" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E109" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>4</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="4" t="s">
         <v>114</v>
       </c>
       <c r="C110" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E110" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>5</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="4" t="s">
         <v>115</v>
       </c>
       <c r="C111" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E111" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>6</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="4" t="s">
         <v>116</v>
       </c>
       <c r="C112" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E112" t="s">
-        <v>216</v>
+        <v>323</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>7</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B113" s="4" t="s">
         <v>117</v>
       </c>
       <c r="C113" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E113" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>8</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="4" t="s">
         <v>118</v>
       </c>
       <c r="C114" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E114" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>9</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="4" t="s">
         <v>119</v>
       </c>
       <c r="C115" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E115" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>10</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="4" t="s">
         <v>120</v>
       </c>
       <c r="C116" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E116" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>11</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="4" t="s">
         <v>121</v>
       </c>
       <c r="C117" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E117" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>12</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="4" t="s">
         <v>122</v>
       </c>
       <c r="C118" t="s">
-        <v>272</v>
-      </c>
-      <c r="E118">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>13</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="4" t="s">
         <v>123</v>
       </c>
       <c r="C119" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E119" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>14</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="4" t="s">
         <v>124</v>
       </c>
       <c r="C120" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E120" t="s">
-        <v>246</v>
+        <v>327</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>15</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="4" t="s">
         <v>125</v>
       </c>
       <c r="C121" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E121" t="s">
-        <v>247</v>
+        <v>229</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>16</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="4" t="s">
         <v>126</v>
       </c>
       <c r="C122" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E122" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>17</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="4" t="s">
         <v>127</v>
       </c>
       <c r="C123" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E123" t="s">
-        <v>174</v>
+        <v>320</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>18</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="4" t="s">
         <v>128</v>
       </c>
       <c r="C124" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E124" t="s">
-        <v>248</v>
+        <v>230</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>19</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="4" t="s">
         <v>129</v>
       </c>
       <c r="C125" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E125" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>20</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="4" t="s">
         <v>130</v>
       </c>
       <c r="C126" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E126" t="s">
-        <v>249</v>
+        <v>231</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>21</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="4" t="s">
         <v>131</v>
       </c>
       <c r="C127" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>22</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="4" t="s">
         <v>132</v>
       </c>
       <c r="C128" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E128" t="s">
-        <v>250</v>
+        <v>232</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>23</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="4" t="s">
         <v>133</v>
       </c>
       <c r="C129" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E129" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>24</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="4" t="s">
         <v>134</v>
       </c>
       <c r="C130" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E130" t="s">
-        <v>251</v>
+        <v>337</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>25</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="4" t="s">
         <v>135</v>
       </c>
       <c r="C131" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E131" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>26</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="4" t="s">
         <v>136</v>
       </c>
       <c r="C132" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E132" t="s">
-        <v>252</v>
+        <v>233</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>27</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="4" t="s">
         <v>137</v>
       </c>
       <c r="C133" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E133" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>28</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="4" t="s">
         <v>138</v>
       </c>
       <c r="C134" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E134" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>29</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="4" t="s">
         <v>139</v>
       </c>
       <c r="C135" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E135" t="s">
-        <v>254</v>
+        <v>235</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>30</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B136" s="4" t="s">
         <v>140</v>
       </c>
       <c r="C136" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="E136" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>1</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B137" s="4" t="s">
         <v>141</v>
       </c>
       <c r="C137" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E137" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>2</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B138" s="4" t="s">
         <v>142</v>
       </c>
       <c r="C138" t="s">
-        <v>273</v>
-      </c>
-      <c r="E138" s="2">
-        <v>45748</v>
+        <v>252</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>3</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B139" s="4" t="s">
         <v>143</v>
       </c>
       <c r="C139" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E139" t="s">
-        <v>257</v>
+        <v>238</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>4</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B140" s="4" t="s">
         <v>144</v>
       </c>
       <c r="C140" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E140" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>5</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B141" s="4" t="s">
         <v>145</v>
       </c>
       <c r="C141" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E141" t="s">
         <v>173</v>
@@ -3171,201 +3423,201 @@
       <c r="A142">
         <v>6</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B142" s="4" t="s">
         <v>146</v>
       </c>
       <c r="C142" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>7</v>
       </c>
-      <c r="B143" t="s">
+      <c r="B143" s="4" t="s">
         <v>147</v>
       </c>
       <c r="C143" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E143" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>8</v>
       </c>
-      <c r="B144" t="s">
+      <c r="B144" s="4" t="s">
         <v>148</v>
       </c>
       <c r="C144" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E144" t="s">
-        <v>259</v>
+        <v>240</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>9</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B145" s="4" t="s">
         <v>149</v>
       </c>
       <c r="C145" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E145" t="s">
-        <v>260</v>
+        <v>241</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>10</v>
       </c>
-      <c r="B146" t="s">
+      <c r="B146" s="4" t="s">
         <v>150</v>
       </c>
       <c r="C146" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E146" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>11</v>
       </c>
-      <c r="B147" t="s">
+      <c r="B147" s="4" t="s">
         <v>151</v>
       </c>
       <c r="C147" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E147" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>12</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B148" s="4" t="s">
         <v>152</v>
       </c>
       <c r="C148" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E148" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>13</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B149" s="4" t="s">
         <v>153</v>
       </c>
       <c r="C149" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E149" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>14</v>
       </c>
-      <c r="B150" t="s">
+      <c r="B150" s="4" t="s">
         <v>154</v>
       </c>
       <c r="C150" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>15</v>
       </c>
-      <c r="B151" t="s">
+      <c r="B151" s="4" t="s">
         <v>155</v>
       </c>
       <c r="C151" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E151" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>16</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B152" s="4" t="s">
         <v>156</v>
       </c>
       <c r="C152" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E152" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>17</v>
       </c>
-      <c r="B153" t="s">
+      <c r="B153" s="4" t="s">
         <v>157</v>
       </c>
       <c r="C153" t="s">
-        <v>273</v>
-      </c>
-      <c r="E153" t="s">
-        <v>209</v>
+        <v>252</v>
+      </c>
+      <c r="E153" s="9">
+        <v>45748</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>18</v>
       </c>
-      <c r="B154" t="s">
+      <c r="B154" s="4" t="s">
         <v>158</v>
       </c>
       <c r="C154" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E154" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>19</v>
       </c>
-      <c r="B155" t="s">
+      <c r="B155" s="4" t="s">
         <v>159</v>
       </c>
       <c r="C155" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E155" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>20</v>
       </c>
-      <c r="B156" t="s">
+      <c r="B156" s="4" t="s">
         <v>160</v>
       </c>
       <c r="C156" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E156" t="s">
         <v>173</v>
@@ -3375,64 +3627,64 @@
       <c r="A157">
         <v>21</v>
       </c>
-      <c r="B157" t="s">
+      <c r="B157" s="4" t="s">
         <v>161</v>
       </c>
       <c r="C157" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>22</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B158" s="4" t="s">
         <v>162</v>
       </c>
       <c r="C158" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E158" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>23</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B159" s="4" t="s">
         <v>163</v>
       </c>
       <c r="C159" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E159" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>24</v>
       </c>
-      <c r="B160" t="s">
+      <c r="B160" s="4" t="s">
         <v>164</v>
       </c>
       <c r="C160" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E160" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>25</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B161" s="4" t="s">
         <v>165</v>
       </c>
       <c r="C161" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E161">
         <v>2024</v>
@@ -3442,67 +3694,672 @@
       <c r="A162">
         <v>26</v>
       </c>
-      <c r="B162" t="s">
+      <c r="B162" s="4" t="s">
         <v>166</v>
       </c>
       <c r="C162" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E162" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>27</v>
       </c>
-      <c r="B163" t="s">
+      <c r="B163" s="4" t="s">
         <v>167</v>
       </c>
       <c r="C163" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E163" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>28</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B164" s="4" t="s">
         <v>168</v>
       </c>
       <c r="C164" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="E164" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>29</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B165" s="4" t="s">
         <v>169</v>
       </c>
       <c r="C165" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>30</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B166" s="4" t="s">
         <v>170</v>
       </c>
       <c r="C166" t="s">
+        <v>252</v>
+      </c>
+      <c r="E166" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B167" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="C167" t="s">
+        <v>252</v>
+      </c>
+      <c r="E167" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B168" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C168" t="s">
+        <v>252</v>
+      </c>
+      <c r="E168" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B169" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C169" t="s">
+        <v>252</v>
+      </c>
+      <c r="E169" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B170" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C170" t="s">
+        <v>252</v>
+      </c>
+      <c r="E170" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B171" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="C171" t="s">
+        <v>252</v>
+      </c>
+      <c r="E171" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B172" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="C172" t="s">
+        <v>252</v>
+      </c>
+      <c r="E172" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B173" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="C173" t="s">
+        <v>252</v>
+      </c>
+      <c r="E173" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B174" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C174" t="s">
+        <v>252</v>
+      </c>
+      <c r="E174" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B175" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="C175" t="s">
+        <v>252</v>
+      </c>
+      <c r="E175" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B176" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="C176" t="s">
+        <v>252</v>
+      </c>
+      <c r="E176" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="177" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B177" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="E166" t="s">
+      <c r="C177" t="s">
+        <v>272</v>
+      </c>
+      <c r="E177" s="7" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="178" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B178" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="C178" t="s">
+        <v>272</v>
+      </c>
+      <c r="E178" s="7" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="179" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B179" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="C179" t="s">
+        <v>272</v>
+      </c>
+      <c r="E179" s="7" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="180" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B180" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C180" t="s">
+        <v>272</v>
+      </c>
+      <c r="E180" s="7" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="181" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B181" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="C181" t="s">
+        <v>272</v>
+      </c>
+      <c r="E181" s="8" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="182" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B182" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="C182" t="s">
+        <v>272</v>
+      </c>
+      <c r="E182" s="8" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="183" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B183" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="C183" t="s">
+        <v>272</v>
+      </c>
+      <c r="E183" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="184" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B184" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="C184" t="s">
+        <v>272</v>
+      </c>
+      <c r="E184" s="8" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="185" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B185" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="C185" t="s">
+        <v>272</v>
+      </c>
+      <c r="E185" s="8" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="186" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B186" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="C186" t="s">
+        <v>272</v>
+      </c>
+      <c r="E186" s="8" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="187" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B187" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="C187" t="s">
+        <v>272</v>
+      </c>
+      <c r="E187" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="188" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B188" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="C188" t="s">
+        <v>272</v>
+      </c>
+      <c r="E188" s="8" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="189" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B189" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C189" t="s">
+        <v>272</v>
+      </c>
+      <c r="E189" s="8" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="190" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B190" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="C190" t="s">
+        <v>272</v>
+      </c>
+      <c r="E190" s="8" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="191" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B191" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="C191" t="s">
+        <v>272</v>
+      </c>
+      <c r="E191" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="192" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B192" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="C192" t="s">
+        <v>272</v>
+      </c>
+      <c r="E192" s="7" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="193" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B193" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="C193" t="s">
+        <v>272</v>
+      </c>
+      <c r="E193" s="7" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="194" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B194" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C194" t="s">
+        <v>272</v>
+      </c>
+      <c r="E194" s="7"/>
+    </row>
+    <row r="195" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B195" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="C195" t="s">
+        <v>272</v>
+      </c>
+      <c r="E195" s="7" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="196" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B196" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="C196" t="s">
+        <v>272</v>
+      </c>
+      <c r="E196" s="8" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="197" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B197" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="C197" t="s">
+        <v>272</v>
+      </c>
+      <c r="E197" s="7" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="198" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B198" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="C198" t="s">
+        <v>272</v>
+      </c>
+      <c r="E198" s="7" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="199" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B199" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="C199" t="s">
+        <v>272</v>
+      </c>
+      <c r="E199" s="7"/>
+    </row>
+    <row r="200" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B200" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="C200" t="s">
+        <v>272</v>
+      </c>
+      <c r="E200" s="7" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="201" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B201" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="C201" t="s">
+        <v>272</v>
+      </c>
+      <c r="E201" s="7" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="202" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B202" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="C202" t="s">
+        <v>272</v>
+      </c>
+      <c r="E202" s="7" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="203" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B203" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="C203" t="s">
+        <v>272</v>
+      </c>
+      <c r="E203" s="7" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="204" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B204" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="C204" t="s">
+        <v>272</v>
+      </c>
+      <c r="E204" s="7" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="205" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B205" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="C205" t="s">
+        <v>272</v>
+      </c>
+      <c r="E205" s="7" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="206" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B206" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="C206" t="s">
+        <v>272</v>
+      </c>
+      <c r="E206" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB804D34-6CDD-4CA2-9CBC-1E5B43FEDBED}">
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
         <v>267</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="7">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="7">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" s="7">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" s="7">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" s="7">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="7">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="7">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" s="7">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" s="7">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="7">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" s="7">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="7">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" s="7">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" s="7">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" s="7">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>